<commit_message>
update the counter strike2 data
</commit_message>
<xml_diff>
--- a/datasets/xlsx/CSFaceit.xlsx
+++ b/datasets/xlsx/CSFaceit.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\avery\OneDrive\Desktop\Programming SHit\HardWareWebsite\datasets\xlsx\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{103916BC-7F9A-4919-B90C-221C3DA27004}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8AA6694E-AA9A-4429-BB36-BFF69B7CB495}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-24120" yWindow="-120" windowWidth="24240" windowHeight="13140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="38280" yWindow="7860" windowWidth="24240" windowHeight="13140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Main" sheetId="1" r:id="rId1"/>
@@ -244,7 +244,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2364" uniqueCount="116">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2463" uniqueCount="117">
   <si>
     <t>ID</t>
   </si>
@@ -592,6 +592,9 @@
   </si>
   <si>
     <t>Haven't played FaceIt in too long. We got Overpass and Anubis back in the pool, plus Cache as a bonus. Season 8 also started a bit ago, so Placement matches for that.</t>
+  </si>
+  <si>
+    <t>Cache</t>
   </si>
 </sst>
 </file>
@@ -995,7 +998,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AI337"/>
+  <dimension ref="A1:AI361"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6.42578125" customWidth="1"/>
@@ -31575,8 +31578,69 @@
       </c>
     </row>
     <row r="331" spans="1:35" x14ac:dyDescent="0.25">
-      <c r="B331" s="1"/>
-      <c r="D331" s="2"/>
+      <c r="A331">
+        <v>330</v>
+      </c>
+      <c r="B331" s="1">
+        <v>46253</v>
+      </c>
+      <c r="C331" s="2">
+        <v>0.74791666666666667</v>
+      </c>
+      <c r="D331" s="2">
+        <v>0.74791666666666667</v>
+      </c>
+      <c r="E331" t="s">
+        <v>53</v>
+      </c>
+      <c r="F331" t="s">
+        <v>109</v>
+      </c>
+      <c r="G331" t="s">
+        <v>83</v>
+      </c>
+      <c r="H331" t="s">
+        <v>65</v>
+      </c>
+      <c r="I331" t="s">
+        <v>81</v>
+      </c>
+      <c r="J331" t="s">
+        <v>63</v>
+      </c>
+      <c r="K331">
+        <v>7</v>
+      </c>
+      <c r="L331">
+        <v>4</v>
+      </c>
+      <c r="M331">
+        <v>11</v>
+      </c>
+      <c r="N331">
+        <v>9</v>
+      </c>
+      <c r="O331">
+        <v>1</v>
+      </c>
+      <c r="P331">
+        <v>1</v>
+      </c>
+      <c r="R331">
+        <v>70</v>
+      </c>
+      <c r="T331" t="s">
+        <v>65</v>
+      </c>
+      <c r="U331" t="s">
+        <v>113</v>
+      </c>
+      <c r="V331">
+        <v>1</v>
+      </c>
+      <c r="W331">
+        <v>1.4</v>
+      </c>
       <c r="AA331">
         <f t="shared" si="29"/>
         <v>0</v>
@@ -31591,22 +31655,90 @@
       </c>
       <c r="AE331">
         <f t="shared" si="32"/>
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="332" spans="1:35" x14ac:dyDescent="0.25">
-      <c r="D332" s="2"/>
+      <c r="A332">
+        <v>331</v>
+      </c>
+      <c r="B332" s="1">
+        <v>46261</v>
+      </c>
+      <c r="C332" s="2">
+        <v>0.8041666666666667</v>
+      </c>
+      <c r="D332" s="2">
+        <v>0.8041666666666667</v>
+      </c>
+      <c r="E332" t="s">
+        <v>61</v>
+      </c>
+      <c r="F332" t="s">
+        <v>107</v>
+      </c>
+      <c r="G332" t="s">
+        <v>83</v>
+      </c>
+      <c r="H332" t="s">
+        <v>65</v>
+      </c>
+      <c r="I332" t="s">
+        <v>116</v>
+      </c>
+      <c r="J332" t="s">
+        <v>55</v>
+      </c>
+      <c r="K332">
+        <v>2</v>
+      </c>
+      <c r="L332">
+        <v>1</v>
+      </c>
+      <c r="M332">
+        <v>6</v>
+      </c>
+      <c r="N332">
+        <v>7</v>
+      </c>
+      <c r="O332">
+        <v>4</v>
+      </c>
+      <c r="P332">
+        <v>8</v>
+      </c>
+      <c r="Q332">
+        <v>1162</v>
+      </c>
+      <c r="R332">
+        <v>64</v>
+      </c>
+      <c r="S332">
+        <v>33</v>
+      </c>
+      <c r="T332" t="s">
+        <v>56</v>
+      </c>
+      <c r="U332" t="s">
+        <v>113</v>
+      </c>
+      <c r="V332">
+        <v>1</v>
+      </c>
+      <c r="W332">
+        <v>0.81</v>
+      </c>
       <c r="AA332">
         <f t="shared" si="29"/>
         <v>0</v>
       </c>
       <c r="AC332">
         <f t="shared" si="30"/>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AD332">
         <f t="shared" si="31"/>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AE332">
         <f t="shared" si="32"/>
@@ -31614,14 +31746,82 @@
       </c>
     </row>
     <row r="333" spans="1:35" x14ac:dyDescent="0.25">
-      <c r="D333" s="2"/>
+      <c r="A333">
+        <v>332</v>
+      </c>
+      <c r="B333" s="1">
+        <v>46261</v>
+      </c>
+      <c r="C333" s="2">
+        <v>0.8354166666666667</v>
+      </c>
+      <c r="D333" s="2">
+        <v>0.8354166666666667</v>
+      </c>
+      <c r="E333" t="s">
+        <v>61</v>
+      </c>
+      <c r="F333" t="s">
+        <v>109</v>
+      </c>
+      <c r="G333" t="s">
+        <v>83</v>
+      </c>
+      <c r="H333" t="s">
+        <v>56</v>
+      </c>
+      <c r="I333" t="s">
+        <v>64</v>
+      </c>
+      <c r="J333" t="s">
+        <v>63</v>
+      </c>
+      <c r="K333">
+        <v>14</v>
+      </c>
+      <c r="L333">
+        <v>3</v>
+      </c>
+      <c r="M333">
+        <v>7</v>
+      </c>
+      <c r="N333">
+        <v>9</v>
+      </c>
+      <c r="O333">
+        <v>2</v>
+      </c>
+      <c r="P333">
+        <v>4</v>
+      </c>
+      <c r="R333">
+        <v>106</v>
+      </c>
+      <c r="S333">
+        <v>34</v>
+      </c>
+      <c r="T333" t="s">
+        <v>65</v>
+      </c>
+      <c r="U333" t="s">
+        <v>113</v>
+      </c>
+      <c r="V333">
+        <v>1</v>
+      </c>
+      <c r="W333">
+        <v>1.8</v>
+      </c>
+      <c r="X333">
+        <v>49</v>
+      </c>
       <c r="AA333">
         <f t="shared" si="29"/>
         <v>0</v>
       </c>
       <c r="AC333">
         <f t="shared" si="30"/>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AD333">
         <f t="shared" si="31"/>
@@ -31629,18 +31829,83 @@
       </c>
       <c r="AE333">
         <f t="shared" si="32"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="334" spans="1:35" x14ac:dyDescent="0.25">
-      <c r="D334" s="2"/>
+      <c r="A334">
+        <v>333</v>
+      </c>
+      <c r="B334" s="1">
+        <v>46265</v>
+      </c>
+      <c r="C334" s="2">
+        <v>0.9375</v>
+      </c>
+      <c r="D334" s="2">
+        <v>0.9375</v>
+      </c>
+      <c r="E334" t="s">
+        <v>53</v>
+      </c>
+      <c r="F334" t="s">
+        <v>106</v>
+      </c>
+      <c r="G334" t="s">
+        <v>89</v>
+      </c>
+      <c r="H334" t="s">
+        <v>56</v>
+      </c>
+      <c r="I334" t="s">
+        <v>62</v>
+      </c>
+      <c r="J334" t="s">
+        <v>63</v>
+      </c>
+      <c r="K334">
+        <v>7</v>
+      </c>
+      <c r="L334">
+        <v>2</v>
+      </c>
+      <c r="M334">
+        <v>9</v>
+      </c>
+      <c r="N334">
+        <v>3</v>
+      </c>
+      <c r="O334">
+        <v>3</v>
+      </c>
+      <c r="P334">
+        <v>4</v>
+      </c>
+      <c r="R334">
+        <v>67</v>
+      </c>
+      <c r="S334">
+        <v>50</v>
+      </c>
+      <c r="T334" t="s">
+        <v>65</v>
+      </c>
+      <c r="U334" t="s">
+        <v>113</v>
+      </c>
+      <c r="V334">
+        <v>2</v>
+      </c>
+      <c r="W334">
+        <v>1.1000000000000001</v>
+      </c>
       <c r="AA334">
         <f t="shared" si="29"/>
         <v>0</v>
       </c>
       <c r="AC334">
         <f t="shared" si="30"/>
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="AD334">
         <f t="shared" si="31"/>
@@ -31648,18 +31913,89 @@
       </c>
       <c r="AE334">
         <f t="shared" si="32"/>
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="335" spans="1:35" x14ac:dyDescent="0.25">
-      <c r="D335" s="2"/>
+      <c r="A335">
+        <v>334</v>
+      </c>
+      <c r="B335" s="1">
+        <v>46265</v>
+      </c>
+      <c r="C335" s="2">
+        <v>0.98750000000000004</v>
+      </c>
+      <c r="D335" s="2">
+        <v>0.98750000000000004</v>
+      </c>
+      <c r="E335" t="s">
+        <v>53</v>
+      </c>
+      <c r="F335" t="s">
+        <v>109</v>
+      </c>
+      <c r="G335" t="s">
+        <v>83</v>
+      </c>
+      <c r="H335" t="s">
+        <v>65</v>
+      </c>
+      <c r="I335" t="s">
+        <v>81</v>
+      </c>
+      <c r="J335" t="s">
+        <v>55</v>
+      </c>
+      <c r="K335">
+        <v>12</v>
+      </c>
+      <c r="L335">
+        <v>4</v>
+      </c>
+      <c r="M335">
+        <v>7</v>
+      </c>
+      <c r="N335">
+        <v>6</v>
+      </c>
+      <c r="O335">
+        <v>4</v>
+      </c>
+      <c r="P335">
+        <v>8</v>
+      </c>
+      <c r="Q335">
+        <v>2105</v>
+      </c>
+      <c r="R335">
+        <v>87</v>
+      </c>
+      <c r="S335">
+        <v>22</v>
+      </c>
+      <c r="T335" t="s">
+        <v>65</v>
+      </c>
+      <c r="U335" t="s">
+        <v>113</v>
+      </c>
+      <c r="V335">
+        <v>1</v>
+      </c>
+      <c r="W335">
+        <v>1.19</v>
+      </c>
+      <c r="X335">
+        <v>49</v>
+      </c>
       <c r="AA335">
         <f t="shared" si="29"/>
         <v>0</v>
       </c>
       <c r="AC335">
         <f t="shared" si="30"/>
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="AD335">
         <f t="shared" si="31"/>
@@ -31667,44 +32003,988 @@
       </c>
       <c r="AE335">
         <f t="shared" si="32"/>
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="336" spans="1:35" x14ac:dyDescent="0.25">
-      <c r="D336" s="2"/>
+      <c r="A336">
+        <v>335</v>
+      </c>
+      <c r="B336" s="1">
+        <v>46274</v>
+      </c>
+      <c r="C336" s="2">
+        <v>0.87638888888888888</v>
+      </c>
+      <c r="D336" s="2">
+        <v>0.87638888888888888</v>
+      </c>
+      <c r="E336" t="s">
+        <v>53</v>
+      </c>
+      <c r="F336" t="s">
+        <v>106</v>
+      </c>
+      <c r="G336" t="s">
+        <v>83</v>
+      </c>
+      <c r="H336" t="s">
+        <v>56</v>
+      </c>
+      <c r="I336" t="s">
+        <v>64</v>
+      </c>
+      <c r="J336" t="s">
+        <v>63</v>
+      </c>
+      <c r="K336">
+        <v>7</v>
+      </c>
+      <c r="L336">
+        <v>0</v>
+      </c>
+      <c r="M336">
+        <v>10</v>
+      </c>
+      <c r="N336">
+        <v>3</v>
+      </c>
+      <c r="O336">
+        <v>0</v>
+      </c>
+      <c r="P336">
+        <v>4</v>
+      </c>
+      <c r="Q336">
+        <v>1129</v>
+      </c>
+      <c r="R336">
+        <v>65</v>
+      </c>
+      <c r="S336">
+        <v>30</v>
+      </c>
+      <c r="T336" t="s">
+        <v>56</v>
+      </c>
+      <c r="U336" t="s">
+        <v>113</v>
+      </c>
+      <c r="V336">
+        <v>2</v>
+      </c>
       <c r="AA336">
         <f t="shared" si="29"/>
         <v>0</v>
       </c>
       <c r="AC336">
         <f t="shared" si="30"/>
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="AD336">
         <f t="shared" si="31"/>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AE336">
         <f t="shared" si="32"/>
         <v>0</v>
       </c>
     </row>
-    <row r="337" spans="4:31" x14ac:dyDescent="0.25">
-      <c r="D337" s="2"/>
+    <row r="337" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A337">
+        <v>336</v>
+      </c>
+      <c r="B337" s="1">
+        <v>46274</v>
+      </c>
+      <c r="C337" s="2">
+        <v>0.89583333333333337</v>
+      </c>
+      <c r="D337" s="2">
+        <v>0.89583333333333337</v>
+      </c>
+      <c r="E337" t="s">
+        <v>53</v>
+      </c>
+      <c r="F337" t="s">
+        <v>106</v>
+      </c>
+      <c r="G337" t="s">
+        <v>83</v>
+      </c>
+      <c r="H337" t="s">
+        <v>56</v>
+      </c>
+      <c r="I337" t="s">
+        <v>79</v>
+      </c>
+      <c r="J337" t="s">
+        <v>63</v>
+      </c>
+      <c r="K337">
+        <v>9</v>
+      </c>
+      <c r="L337">
+        <v>2</v>
+      </c>
+      <c r="M337">
+        <v>9</v>
+      </c>
+      <c r="N337">
+        <v>4</v>
+      </c>
+      <c r="P337">
+        <v>5</v>
+      </c>
+      <c r="T337" t="s">
+        <v>56</v>
+      </c>
+      <c r="U337" t="s">
+        <v>113</v>
+      </c>
+      <c r="V337">
+        <v>2</v>
+      </c>
       <c r="AA337">
         <f t="shared" si="29"/>
         <v>0</v>
       </c>
       <c r="AC337">
         <f t="shared" si="30"/>
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="AD337">
         <f t="shared" si="31"/>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AE337">
         <f t="shared" si="32"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="338" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A338">
+        <v>337</v>
+      </c>
+      <c r="B338" s="1">
+        <v>46275</v>
+      </c>
+      <c r="C338" s="2">
+        <v>9.0277777777777769E-3</v>
+      </c>
+      <c r="D338" s="2">
+        <v>9.0277777777777769E-3</v>
+      </c>
+      <c r="E338" s="2"/>
+      <c r="F338" t="s">
+        <v>109</v>
+      </c>
+      <c r="G338" t="s">
+        <v>83</v>
+      </c>
+      <c r="H338" t="s">
+        <v>65</v>
+      </c>
+      <c r="I338" t="s">
+        <v>62</v>
+      </c>
+      <c r="J338" t="s">
+        <v>55</v>
+      </c>
+      <c r="K338">
+        <v>9</v>
+      </c>
+      <c r="L338">
+        <v>3</v>
+      </c>
+      <c r="M338">
+        <v>10</v>
+      </c>
+      <c r="N338">
+        <v>5</v>
+      </c>
+      <c r="O338">
+        <v>3</v>
+      </c>
+      <c r="P338">
+        <v>5</v>
+      </c>
+      <c r="R338">
+        <v>54</v>
+      </c>
+      <c r="S338">
+        <v>35</v>
+      </c>
+      <c r="T338" t="s">
+        <v>65</v>
+      </c>
+      <c r="U338" t="s">
+        <v>113</v>
+      </c>
+      <c r="V338">
+        <v>1</v>
+      </c>
+      <c r="W338">
+        <v>1.08</v>
+      </c>
+      <c r="AA338">
+        <f t="shared" ref="AA338:AA361" si="34">(Y338+Z338)/2</f>
+        <v>0</v>
+      </c>
+      <c r="AC338">
+        <f t="shared" ref="AC338:AC361" si="35">IF(B338=B337, AC337+1, 1)</f>
+        <v>1</v>
+      </c>
+      <c r="AD338">
+        <f t="shared" ref="AD338:AD361" si="36">IF(T338="Loss",AC337+1,0)</f>
+        <v>0</v>
+      </c>
+      <c r="AE338">
+        <f t="shared" ref="AE338:AE361" si="37">IF(T338="Win",AE337+1,0)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="339" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A339">
+        <v>338</v>
+      </c>
+      <c r="B339" s="1">
+        <v>46275</v>
+      </c>
+      <c r="C339" s="2">
+        <v>0.76875000000000004</v>
+      </c>
+      <c r="D339" s="2">
+        <v>0.76875000000000004</v>
+      </c>
+      <c r="E339" t="s">
+        <v>53</v>
+      </c>
+      <c r="F339" t="s">
+        <v>107</v>
+      </c>
+      <c r="G339" t="s">
+        <v>83</v>
+      </c>
+      <c r="H339" t="s">
+        <v>65</v>
+      </c>
+      <c r="I339" t="s">
+        <v>80</v>
+      </c>
+      <c r="J339" t="s">
+        <v>55</v>
+      </c>
+      <c r="K339">
+        <v>9</v>
+      </c>
+      <c r="L339">
+        <v>1</v>
+      </c>
+      <c r="M339">
+        <v>10</v>
+      </c>
+      <c r="N339">
+        <v>14</v>
+      </c>
+      <c r="O339">
+        <v>2</v>
+      </c>
+      <c r="P339">
+        <v>7</v>
+      </c>
+      <c r="Q339">
+        <v>2226</v>
+      </c>
+      <c r="R339">
+        <v>96</v>
+      </c>
+      <c r="S339">
+        <v>43</v>
+      </c>
+      <c r="T339" t="s">
+        <v>56</v>
+      </c>
+      <c r="U339" t="s">
+        <v>113</v>
+      </c>
+      <c r="V339">
+        <v>1</v>
+      </c>
+      <c r="AA339">
+        <f t="shared" si="34"/>
+        <v>0</v>
+      </c>
+      <c r="AC339">
+        <f t="shared" si="35"/>
+        <v>2</v>
+      </c>
+      <c r="AD339">
+        <f t="shared" si="36"/>
+        <v>2</v>
+      </c>
+      <c r="AE339">
+        <f t="shared" si="37"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="340" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A340">
+        <v>339</v>
+      </c>
+      <c r="B340" s="1">
+        <v>46275</v>
+      </c>
+      <c r="C340" s="2">
+        <v>0.85138888888888886</v>
+      </c>
+      <c r="D340" s="2">
+        <v>0.85138888888888886</v>
+      </c>
+      <c r="E340" t="s">
+        <v>61</v>
+      </c>
+      <c r="F340" t="s">
+        <v>106</v>
+      </c>
+      <c r="G340" t="s">
+        <v>83</v>
+      </c>
+      <c r="H340" t="s">
+        <v>65</v>
+      </c>
+      <c r="I340" t="s">
+        <v>79</v>
+      </c>
+      <c r="J340" t="s">
+        <v>55</v>
+      </c>
+      <c r="K340">
+        <v>5</v>
+      </c>
+      <c r="L340">
+        <v>3</v>
+      </c>
+      <c r="M340">
+        <v>7</v>
+      </c>
+      <c r="N340">
+        <v>6</v>
+      </c>
+      <c r="O340">
+        <v>3</v>
+      </c>
+      <c r="P340">
+        <v>5</v>
+      </c>
+      <c r="R340">
+        <v>54</v>
+      </c>
+      <c r="S340">
+        <v>18</v>
+      </c>
+      <c r="T340" t="s">
+        <v>65</v>
+      </c>
+      <c r="U340">
+        <v>1023</v>
+      </c>
+      <c r="V340">
+        <v>1</v>
+      </c>
+      <c r="W340">
+        <v>1</v>
+      </c>
+      <c r="AA340">
+        <f t="shared" si="34"/>
+        <v>0</v>
+      </c>
+      <c r="AC340">
+        <f t="shared" si="35"/>
+        <v>3</v>
+      </c>
+      <c r="AD340">
+        <f t="shared" si="36"/>
+        <v>0</v>
+      </c>
+      <c r="AE340">
+        <f t="shared" si="37"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="341" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A341">
+        <v>340</v>
+      </c>
+      <c r="B341" s="1">
+        <v>46275</v>
+      </c>
+      <c r="C341" s="2">
+        <v>0.91805555555555551</v>
+      </c>
+      <c r="D341" s="2">
+        <v>0.91805555555555551</v>
+      </c>
+      <c r="E341" t="s">
+        <v>53</v>
+      </c>
+      <c r="F341" t="s">
+        <v>107</v>
+      </c>
+      <c r="G341" t="s">
+        <v>83</v>
+      </c>
+      <c r="H341" t="s">
+        <v>65</v>
+      </c>
+      <c r="I341" t="s">
+        <v>79</v>
+      </c>
+      <c r="J341" t="s">
+        <v>55</v>
+      </c>
+      <c r="K341">
+        <v>7</v>
+      </c>
+      <c r="L341">
+        <v>1</v>
+      </c>
+      <c r="M341">
+        <v>9</v>
+      </c>
+      <c r="N341">
+        <v>6</v>
+      </c>
+      <c r="O341">
+        <v>3</v>
+      </c>
+      <c r="P341">
+        <v>8</v>
+      </c>
+      <c r="R341">
+        <v>77</v>
+      </c>
+      <c r="T341" t="s">
+        <v>65</v>
+      </c>
+      <c r="U341">
+        <v>1047</v>
+      </c>
+      <c r="V341">
+        <v>1</v>
+      </c>
+      <c r="W341">
+        <v>0.96</v>
+      </c>
+      <c r="AA341">
+        <f t="shared" si="34"/>
+        <v>0</v>
+      </c>
+      <c r="AC341">
+        <f t="shared" si="35"/>
+        <v>4</v>
+      </c>
+      <c r="AD341">
+        <f t="shared" si="36"/>
+        <v>0</v>
+      </c>
+      <c r="AE341">
+        <f t="shared" si="37"/>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="342" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A342">
+        <v>341</v>
+      </c>
+      <c r="B342" s="1">
+        <v>46275</v>
+      </c>
+      <c r="C342" s="2">
+        <v>0.95416666666666672</v>
+      </c>
+      <c r="D342" s="2">
+        <v>0.95416666666666672</v>
+      </c>
+      <c r="E342" t="s">
+        <v>61</v>
+      </c>
+      <c r="F342" t="s">
+        <v>109</v>
+      </c>
+      <c r="G342" t="s">
+        <v>83</v>
+      </c>
+      <c r="H342" t="s">
+        <v>56</v>
+      </c>
+      <c r="I342" t="s">
+        <v>62</v>
+      </c>
+      <c r="J342" t="s">
+        <v>63</v>
+      </c>
+      <c r="K342">
+        <v>9</v>
+      </c>
+      <c r="L342">
+        <v>3</v>
+      </c>
+      <c r="M342">
+        <v>10</v>
+      </c>
+      <c r="N342">
+        <v>6</v>
+      </c>
+      <c r="O342">
+        <v>2</v>
+      </c>
+      <c r="P342">
+        <v>5</v>
+      </c>
+      <c r="T342" t="s">
+        <v>56</v>
+      </c>
+      <c r="U342">
+        <v>1069</v>
+      </c>
+      <c r="V342">
+        <v>1</v>
+      </c>
+      <c r="AA342">
+        <f t="shared" si="34"/>
+        <v>0</v>
+      </c>
+      <c r="AC342">
+        <f t="shared" si="35"/>
+        <v>5</v>
+      </c>
+      <c r="AD342">
+        <f t="shared" si="36"/>
+        <v>5</v>
+      </c>
+      <c r="AE342">
+        <f t="shared" si="37"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="343" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A343">
+        <v>342</v>
+      </c>
+      <c r="B343" s="1">
+        <v>46275</v>
+      </c>
+      <c r="C343" s="2">
+        <v>0.97916666666666663</v>
+      </c>
+      <c r="D343" s="2">
+        <v>0.97916666666666663</v>
+      </c>
+      <c r="E343" t="s">
+        <v>61</v>
+      </c>
+      <c r="F343" t="s">
+        <v>106</v>
+      </c>
+      <c r="G343" t="s">
+        <v>83</v>
+      </c>
+      <c r="H343" t="s">
+        <v>65</v>
+      </c>
+      <c r="I343" t="s">
+        <v>81</v>
+      </c>
+      <c r="J343" t="s">
+        <v>55</v>
+      </c>
+      <c r="K343">
+        <v>2</v>
+      </c>
+      <c r="L343">
+        <v>2</v>
+      </c>
+      <c r="M343">
+        <v>9</v>
+      </c>
+      <c r="N343">
+        <v>4</v>
+      </c>
+      <c r="O343">
+        <v>5</v>
+      </c>
+      <c r="P343">
+        <v>7</v>
+      </c>
+      <c r="R343">
+        <v>58</v>
+      </c>
+      <c r="S343">
+        <v>36</v>
+      </c>
+      <c r="T343" t="s">
+        <v>56</v>
+      </c>
+      <c r="U343">
+        <v>1047</v>
+      </c>
+      <c r="V343">
+        <v>1</v>
+      </c>
+      <c r="W343">
+        <v>0.76</v>
+      </c>
+      <c r="AA343">
+        <f t="shared" si="34"/>
+        <v>0</v>
+      </c>
+      <c r="AC343">
+        <f t="shared" si="35"/>
+        <v>6</v>
+      </c>
+      <c r="AD343">
+        <f t="shared" si="36"/>
+        <v>6</v>
+      </c>
+      <c r="AE343">
+        <f t="shared" si="37"/>
+        <v>0</v>
+      </c>
+      <c r="AF343">
+        <v>-4.84</v>
+      </c>
+      <c r="AG343">
+        <v>30</v>
+      </c>
+      <c r="AH343">
+        <v>44</v>
+      </c>
+      <c r="AI343">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="344" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="AA344">
+        <f t="shared" si="34"/>
+        <v>0</v>
+      </c>
+      <c r="AC344">
+        <f t="shared" si="35"/>
+        <v>1</v>
+      </c>
+      <c r="AD344">
+        <f t="shared" si="36"/>
+        <v>0</v>
+      </c>
+      <c r="AE344">
+        <f t="shared" si="37"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="345" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="AA345">
+        <f t="shared" si="34"/>
+        <v>0</v>
+      </c>
+      <c r="AC345">
+        <f t="shared" si="35"/>
+        <v>2</v>
+      </c>
+      <c r="AD345">
+        <f t="shared" si="36"/>
+        <v>0</v>
+      </c>
+      <c r="AE345">
+        <f t="shared" si="37"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="346" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="AA346">
+        <f t="shared" si="34"/>
+        <v>0</v>
+      </c>
+      <c r="AC346">
+        <f t="shared" si="35"/>
+        <v>3</v>
+      </c>
+      <c r="AD346">
+        <f t="shared" si="36"/>
+        <v>0</v>
+      </c>
+      <c r="AE346">
+        <f t="shared" si="37"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="347" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="AA347">
+        <f t="shared" si="34"/>
+        <v>0</v>
+      </c>
+      <c r="AC347">
+        <f t="shared" si="35"/>
+        <v>4</v>
+      </c>
+      <c r="AD347">
+        <f t="shared" si="36"/>
+        <v>0</v>
+      </c>
+      <c r="AE347">
+        <f t="shared" si="37"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="348" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="AA348">
+        <f t="shared" si="34"/>
+        <v>0</v>
+      </c>
+      <c r="AC348">
+        <f t="shared" si="35"/>
+        <v>5</v>
+      </c>
+      <c r="AD348">
+        <f t="shared" si="36"/>
+        <v>0</v>
+      </c>
+      <c r="AE348">
+        <f t="shared" si="37"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="349" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="AA349">
+        <f t="shared" si="34"/>
+        <v>0</v>
+      </c>
+      <c r="AC349">
+        <f t="shared" si="35"/>
+        <v>6</v>
+      </c>
+      <c r="AD349">
+        <f t="shared" si="36"/>
+        <v>0</v>
+      </c>
+      <c r="AE349">
+        <f t="shared" si="37"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="350" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="AA350">
+        <f t="shared" si="34"/>
+        <v>0</v>
+      </c>
+      <c r="AC350">
+        <f t="shared" si="35"/>
+        <v>7</v>
+      </c>
+      <c r="AD350">
+        <f t="shared" si="36"/>
+        <v>0</v>
+      </c>
+      <c r="AE350">
+        <f t="shared" si="37"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="351" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="AA351">
+        <f t="shared" si="34"/>
+        <v>0</v>
+      </c>
+      <c r="AC351">
+        <f t="shared" si="35"/>
+        <v>8</v>
+      </c>
+      <c r="AD351">
+        <f t="shared" si="36"/>
+        <v>0</v>
+      </c>
+      <c r="AE351">
+        <f t="shared" si="37"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="352" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="AA352">
+        <f t="shared" si="34"/>
+        <v>0</v>
+      </c>
+      <c r="AC352">
+        <f t="shared" si="35"/>
+        <v>9</v>
+      </c>
+      <c r="AD352">
+        <f t="shared" si="36"/>
+        <v>0</v>
+      </c>
+      <c r="AE352">
+        <f t="shared" si="37"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="353" spans="27:31" x14ac:dyDescent="0.25">
+      <c r="AA353">
+        <f t="shared" si="34"/>
+        <v>0</v>
+      </c>
+      <c r="AC353">
+        <f t="shared" si="35"/>
+        <v>10</v>
+      </c>
+      <c r="AD353">
+        <f t="shared" si="36"/>
+        <v>0</v>
+      </c>
+      <c r="AE353">
+        <f t="shared" si="37"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="354" spans="27:31" x14ac:dyDescent="0.25">
+      <c r="AA354">
+        <f t="shared" si="34"/>
+        <v>0</v>
+      </c>
+      <c r="AC354">
+        <f t="shared" si="35"/>
+        <v>11</v>
+      </c>
+      <c r="AD354">
+        <f t="shared" si="36"/>
+        <v>0</v>
+      </c>
+      <c r="AE354">
+        <f t="shared" si="37"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="355" spans="27:31" x14ac:dyDescent="0.25">
+      <c r="AA355">
+        <f t="shared" si="34"/>
+        <v>0</v>
+      </c>
+      <c r="AC355">
+        <f t="shared" si="35"/>
+        <v>12</v>
+      </c>
+      <c r="AD355">
+        <f t="shared" si="36"/>
+        <v>0</v>
+      </c>
+      <c r="AE355">
+        <f t="shared" si="37"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="356" spans="27:31" x14ac:dyDescent="0.25">
+      <c r="AA356">
+        <f t="shared" si="34"/>
+        <v>0</v>
+      </c>
+      <c r="AC356">
+        <f t="shared" si="35"/>
+        <v>13</v>
+      </c>
+      <c r="AD356">
+        <f t="shared" si="36"/>
+        <v>0</v>
+      </c>
+      <c r="AE356">
+        <f t="shared" si="37"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="357" spans="27:31" x14ac:dyDescent="0.25">
+      <c r="AA357">
+        <f t="shared" si="34"/>
+        <v>0</v>
+      </c>
+      <c r="AC357">
+        <f t="shared" si="35"/>
+        <v>14</v>
+      </c>
+      <c r="AD357">
+        <f t="shared" si="36"/>
+        <v>0</v>
+      </c>
+      <c r="AE357">
+        <f t="shared" si="37"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="358" spans="27:31" x14ac:dyDescent="0.25">
+      <c r="AA358">
+        <f t="shared" si="34"/>
+        <v>0</v>
+      </c>
+      <c r="AC358">
+        <f t="shared" si="35"/>
+        <v>15</v>
+      </c>
+      <c r="AD358">
+        <f t="shared" si="36"/>
+        <v>0</v>
+      </c>
+      <c r="AE358">
+        <f t="shared" si="37"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="359" spans="27:31" x14ac:dyDescent="0.25">
+      <c r="AA359">
+        <f t="shared" si="34"/>
+        <v>0</v>
+      </c>
+      <c r="AC359">
+        <f t="shared" si="35"/>
+        <v>16</v>
+      </c>
+      <c r="AD359">
+        <f t="shared" si="36"/>
+        <v>0</v>
+      </c>
+      <c r="AE359">
+        <f t="shared" si="37"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="360" spans="27:31" x14ac:dyDescent="0.25">
+      <c r="AA360">
+        <f t="shared" si="34"/>
+        <v>0</v>
+      </c>
+      <c r="AC360">
+        <f t="shared" si="35"/>
+        <v>17</v>
+      </c>
+      <c r="AD360">
+        <f t="shared" si="36"/>
+        <v>0</v>
+      </c>
+      <c r="AE360">
+        <f t="shared" si="37"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="361" spans="27:31" x14ac:dyDescent="0.25">
+      <c r="AA361">
+        <f t="shared" si="34"/>
+        <v>0</v>
+      </c>
+      <c r="AC361">
+        <f t="shared" si="35"/>
+        <v>18</v>
+      </c>
+      <c r="AD361">
+        <f t="shared" si="36"/>
+        <v>0</v>
+      </c>
+      <c r="AE361">
+        <f t="shared" si="37"/>
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
errrrrrr, uhhhhhh, data spreadsheet
</commit_message>
<xml_diff>
--- a/datasets/xlsx/CSFaceit.xlsx
+++ b/datasets/xlsx/CSFaceit.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\avery\OneDrive\Desktop\Programming SHit\HardWareWebsite\datasets\xlsx\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8AA6694E-AA9A-4429-BB36-BFF69B7CB495}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1592016E-41F6-4390-8229-B7DCC547E40F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="7860" windowWidth="24240" windowHeight="13140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21240" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Main" sheetId="1" r:id="rId1"/>
@@ -244,7 +244,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2463" uniqueCount="117">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2477" uniqueCount="118">
   <si>
     <t>ID</t>
   </si>
@@ -595,6 +595,9 @@
   </si>
   <si>
     <t>Cache</t>
+  </si>
+  <si>
+    <t>Virginia</t>
   </si>
 </sst>
 </file>
@@ -32665,6 +32668,69 @@
       </c>
     </row>
     <row r="344" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A344">
+        <v>343</v>
+      </c>
+      <c r="B344" s="1">
+        <v>46314</v>
+      </c>
+      <c r="C344" s="2">
+        <v>0.77638888888888891</v>
+      </c>
+      <c r="D344" s="2">
+        <v>0.77638888888888891</v>
+      </c>
+      <c r="E344" t="s">
+        <v>61</v>
+      </c>
+      <c r="F344" t="s">
+        <v>106</v>
+      </c>
+      <c r="G344" t="s">
+        <v>117</v>
+      </c>
+      <c r="H344" t="s">
+        <v>65</v>
+      </c>
+      <c r="I344" t="s">
+        <v>64</v>
+      </c>
+      <c r="J344" t="s">
+        <v>63</v>
+      </c>
+      <c r="K344">
+        <v>12</v>
+      </c>
+      <c r="L344">
+        <v>1</v>
+      </c>
+      <c r="M344">
+        <v>11</v>
+      </c>
+      <c r="N344">
+        <v>9</v>
+      </c>
+      <c r="O344">
+        <v>3</v>
+      </c>
+      <c r="P344">
+        <v>11</v>
+      </c>
+      <c r="Q344">
+        <v>2250</v>
+      </c>
+      <c r="R344">
+        <v>66</v>
+      </c>
+      <c r="T344" t="s">
+        <v>56</v>
+      </c>
+      <c r="U344">
+        <v>1017</v>
+      </c>
+      <c r="V344">
+        <v>1</v>
+      </c>
       <c r="AA344">
         <f t="shared" si="34"/>
         <v>0</v>
@@ -32675,7 +32741,7 @@
       </c>
       <c r="AD344">
         <f t="shared" si="36"/>
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="AE344">
         <f t="shared" si="37"/>
@@ -32683,6 +32749,69 @@
       </c>
     </row>
     <row r="345" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A345">
+        <v>344</v>
+      </c>
+      <c r="B345" s="1">
+        <v>46314</v>
+      </c>
+      <c r="C345" s="2">
+        <v>0.82638888888888884</v>
+      </c>
+      <c r="D345" s="2">
+        <v>0.82638888888888884</v>
+      </c>
+      <c r="E345" t="s">
+        <v>61</v>
+      </c>
+      <c r="F345" t="s">
+        <v>107</v>
+      </c>
+      <c r="G345" t="s">
+        <v>83</v>
+      </c>
+      <c r="H345" t="s">
+        <v>56</v>
+      </c>
+      <c r="I345" t="s">
+        <v>62</v>
+      </c>
+      <c r="J345" t="s">
+        <v>63</v>
+      </c>
+      <c r="K345">
+        <v>6</v>
+      </c>
+      <c r="L345">
+        <v>4</v>
+      </c>
+      <c r="M345">
+        <v>6</v>
+      </c>
+      <c r="N345">
+        <v>6</v>
+      </c>
+      <c r="O345">
+        <v>3</v>
+      </c>
+      <c r="P345">
+        <v>1</v>
+      </c>
+      <c r="Q345">
+        <v>1253</v>
+      </c>
+      <c r="R345">
+        <v>69</v>
+      </c>
+      <c r="T345" t="s">
+        <v>65</v>
+      </c>
+      <c r="U345">
+        <v>993</v>
+      </c>
+      <c r="V345">
+        <v>1</v>
+      </c>
       <c r="AA345">
         <f t="shared" si="34"/>
         <v>0</v>
@@ -32697,7 +32826,7 @@
       </c>
       <c r="AE345">
         <f t="shared" si="37"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="346" spans="1:35" x14ac:dyDescent="0.25">
@@ -32707,7 +32836,7 @@
       </c>
       <c r="AC346">
         <f t="shared" si="35"/>
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AD346">
         <f t="shared" si="36"/>
@@ -32725,7 +32854,7 @@
       </c>
       <c r="AC347">
         <f t="shared" si="35"/>
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="AD347">
         <f t="shared" si="36"/>
@@ -32743,7 +32872,7 @@
       </c>
       <c r="AC348">
         <f t="shared" si="35"/>
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="AD348">
         <f t="shared" si="36"/>
@@ -32761,7 +32890,7 @@
       </c>
       <c r="AC349">
         <f t="shared" si="35"/>
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="AD349">
         <f t="shared" si="36"/>
@@ -32779,7 +32908,7 @@
       </c>
       <c r="AC350">
         <f t="shared" si="35"/>
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="AD350">
         <f t="shared" si="36"/>
@@ -32797,7 +32926,7 @@
       </c>
       <c r="AC351">
         <f t="shared" si="35"/>
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="AD351">
         <f t="shared" si="36"/>
@@ -32815,7 +32944,7 @@
       </c>
       <c r="AC352">
         <f t="shared" si="35"/>
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="AD352">
         <f t="shared" si="36"/>
@@ -32833,7 +32962,7 @@
       </c>
       <c r="AC353">
         <f t="shared" si="35"/>
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="AD353">
         <f t="shared" si="36"/>
@@ -32851,7 +32980,7 @@
       </c>
       <c r="AC354">
         <f t="shared" si="35"/>
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="AD354">
         <f t="shared" si="36"/>
@@ -32869,7 +32998,7 @@
       </c>
       <c r="AC355">
         <f t="shared" si="35"/>
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="AD355">
         <f t="shared" si="36"/>
@@ -32887,7 +33016,7 @@
       </c>
       <c r="AC356">
         <f t="shared" si="35"/>
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="AD356">
         <f t="shared" si="36"/>
@@ -32905,7 +33034,7 @@
       </c>
       <c r="AC357">
         <f t="shared" si="35"/>
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="AD357">
         <f t="shared" si="36"/>
@@ -32923,7 +33052,7 @@
       </c>
       <c r="AC358">
         <f t="shared" si="35"/>
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="AD358">
         <f t="shared" si="36"/>
@@ -32941,7 +33070,7 @@
       </c>
       <c r="AC359">
         <f t="shared" si="35"/>
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="AD359">
         <f t="shared" si="36"/>
@@ -32959,7 +33088,7 @@
       </c>
       <c r="AC360">
         <f t="shared" si="35"/>
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="AD360">
         <f t="shared" si="36"/>
@@ -32977,7 +33106,7 @@
       </c>
       <c r="AC361">
         <f t="shared" si="35"/>
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="AD361">
         <f t="shared" si="36"/>

</xml_diff>